<commit_message>
Test master generation reduction range with historical parameter validation
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/hyperspace_config.xlsx
+++ b/space-battleship/config_excel/hyperspace_config.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C517"/>
+  <dimension ref="A1:C521"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="65" customWidth="1" min="1" max="1"/>
@@ -7489,7 +7489,7 @@
         </is>
       </c>
       <c r="C488" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="489">
@@ -7504,7 +7504,7 @@
         </is>
       </c>
       <c r="C489" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="490">
@@ -7895,6 +7895,63 @@
       </c>
       <c r="C517" t="n">
         <v>600</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>/legendary_effects/drone_master/stored_parameter_ranges</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>/legendary_effects/drone_master/stored_parameter_ranges/maximum_reduction</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="C519" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>/legendary_effects/drone_master/stored_parameter_ranges/maximum_reduction/0</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="C520" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>/legendary_effects/drone_master/stored_parameter_ranges/maximum_reduction/1</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="C521" t="n">
+        <v>0.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Freeze verified final21sheet workbooks with Chinese tuning notes
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/hyperspace_config.xlsx
+++ b/space-battleship/config_excel/hyperspace_config.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础参数" sheetId="1" r:id="Rc2ac7b76d61e4b7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="路线" sheetId="2" r:id="Rbf0e1ed6cde24b59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品质" sheetId="3" r:id="Ra9eadc1285434970"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="舰型容量" sheetId="4" r:id="R0a42e4afc54c47be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶级权重" sheetId="5" r:id="Ra3f0b963ae02477a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="词缀定义" sheetId="6" r:id="R81635538a8934ce0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="词缀区间" sheetId="7" r:id="R5efd77e24aea4c8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="挂设成长" sheetId="8" r:id="Re06f5013d20f40e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="传说定义" sheetId="9" r:id="Racf017048bc84843"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="传说随机参数" sheetId="10" r:id="Rb082764d12b74a63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="传说常量" sheetId="11" r:id="R6fac279790d44201"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改造费用" sheetId="12" r:id="R385ac4f8de9f4c09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定规则_兼容说明" sheetId="13" r:id="Re4fc916136854f26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础参数" sheetId="1" r:id="Rdbf188d28566469a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="路线" sheetId="2" r:id="R07cb589b63f848c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品质" sheetId="3" r:id="R0dd81bc0b9574ae7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="舰型容量" sheetId="4" r:id="R46bfb6ed1af5480e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶级权重" sheetId="5" r:id="R2c3c53182c2d429b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="词缀定义" sheetId="6" r:id="Rbea35f20e078402d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="词缀区间" sheetId="7" r:id="R6447d91b56bb48d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="挂设成长" sheetId="8" r:id="Rad73cc54c5e64ed1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="传说定义" sheetId="9" r:id="Rcc44ca8479a74b8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="传说随机参数" sheetId="10" r:id="R2a9f2c4c89cf47df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="传说常量" sheetId="11" r:id="R19ce7c85c67144c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改造费用" sheetId="12" r:id="Re49bd0df2c8b4b31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定规则_兼容说明" sheetId="13" r:id="Rac066a41c26f4176"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -482,7 +482,7 @@
       <x:c r="A2" s="13" t="str">
         <x:v>现有或本次明确规划的配置键
 单位：稳定ID
-约束：仅已有实现/已验ID；不自动新增功能；非空；主键作用域唯一</x:v>
+约束：仅已有实现/已验ID；不自动新增功能；非空；主键作用域唯一；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="B2" s="13" t="str">
         <x:v>本键固定数据类型，不随单元格显示格式改变
@@ -549,10 +549,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D4" s="19" t="str">
-        <x:v>关</x:v>
+        <x:v>主线最高到达关</x:v>
       </x:c>
       <x:c r="E4" s="19" t="str">
-        <x:v>异空间可用最高到达关卡门槛</x:v>
+        <x:v>默认7。异空间开放门槛。调大更晚开放，调小更早开放；达到门槛仍需满足路线最低关卡和资源条件。正整数，不新增关卡内容。</x:v>
       </x:c>
       <x:c r="F4" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -572,10 +572,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="D5" s="19" t="str">
-        <x:v>关</x:v>
+        <x:v>所选主线等级/关</x:v>
       </x:c>
       <x:c r="E5" s="19" t="str">
-        <x:v>允许探索的最低关卡</x:v>
+        <x:v>默认5。可选择探索的最低主线关。调大屏蔽更多低关，调小允许更早关；所选关不得超过已到达关及正式关卡表。</x:v>
       </x:c>
       <x:c r="F5" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -598,7 +598,7 @@
         <x:v>能量/游戏秒</x:v>
       </x:c>
       <x:c r="E6" s="19" t="str">
-        <x:v>在线游戏时间每秒充能</x:v>
+        <x:v>默认10。在线异空间充能基础速度。调大更快攒票，调小更慢；受挂设及60关后补给倍率共同作用。随游戏时间推进，离线不补充。</x:v>
       </x:c>
       <x:c r="F6" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；&gt;0</x:v>
@@ -621,7 +621,7 @@
         <x:v>能量</x:v>
       </x:c>
       <x:c r="E7" s="19" t="str">
-        <x:v>基础能量容量；自动探索需满容量才派发</x:v>
+        <x:v>默认216000。基础储能上限，也是自动探索满能量派发门槛。调大一次储能更多但首次充满更久，调小更快满；挂设会同步放大容量。</x:v>
       </x:c>
       <x:c r="F7" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；&gt;0</x:v>
@@ -630,7 +630,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="48" customHeight="1">
+    <x:row r="8" ht="62" customHeight="1">
       <x:c r="A8" s="19" t="str">
         <x:v>ticket</x:v>
       </x:c>
@@ -644,7 +644,7 @@
         <x:v>能量/次</x:v>
       </x:c>
       <x:c r="E8" s="19" t="str">
-        <x:v>手动票耗及自动票耗基数；自动再乘船员B/(B+L)，失败退实际已付票</x:v>
+        <x:v>默认108000。手动票耗及自动票耗基数。调大每次消耗更多，调小更便宜；自动再乘B/(B+船员等级)，失败仅退实际已付票。例如B=20、等级20，自动票耗为此值的一半。</x:v>
       </x:c>
       <x:c r="F8" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；&gt;0</x:v>
@@ -653,7 +653,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="48" customHeight="1">
+    <x:row r="9" ht="62" customHeight="1">
       <x:c r="A9" s="19" t="str">
         <x:v>minimum_duration</x:v>
       </x:c>
@@ -667,7 +667,7 @@
         <x:v>游戏秒</x:v>
       </x:c>
       <x:c r="E9" s="19" t="str">
-        <x:v>自动探索最短耗时</x:v>
+        <x:v>默认10。自动探索耗时下限。实际=max(此值,最佳手动X1记录×船员折算)。调大提高最快可达到的耗时下限，调小允许更快；离线不推进。</x:v>
       </x:c>
       <x:c r="F9" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；&gt;0</x:v>
@@ -687,10 +687,10 @@
         <x:v>200</x:v>
       </x:c>
       <x:c r="D10" s="19" t="str">
-        <x:v>格</x:v>
+        <x:v>架/格</x:v>
       </x:c>
       <x:c r="E10" s="19" t="str">
-        <x:v>基础仓库容量</x:v>
+        <x:v>默认200。初始仓库容量。调大能存更多无人机，调小更早满仓；后续容量另加每次重铸增长。影响满仓暂停和领取条件，不直接提升伤害。</x:v>
       </x:c>
       <x:c r="F10" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -699,7 +699,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="22" customHeight="1">
+    <x:row r="11" ht="48" customHeight="1">
       <x:c r="A11" s="19" t="str">
         <x:v>overflow_capacity</x:v>
       </x:c>
@@ -710,10 +710,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D11" s="19" t="str">
-        <x:v>格</x:v>
+        <x:v>架/格</x:v>
       </x:c>
       <x:c r="E11" s="19" t="str">
-        <x:v>固定溢出缓存容量；固定10格</x:v>
+        <x:v>默认10。固定10格溢出缓存，处理正常仓库暂时无法接纳的无人机。只读，必须10，不是可扩容参数。</x:v>
       </x:c>
       <x:c r="F11" s="19" t="str">
         <x:v>必须等于10；只读锁定</x:v>
@@ -733,10 +733,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D12" s="19" t="str">
-        <x:v>格/重铸</x:v>
+        <x:v>格/次重铸</x:v>
       </x:c>
       <x:c r="E12" s="19" t="str">
-        <x:v>每次重铸增加仓库格数</x:v>
+        <x:v>默认10。每次重铸永久增加的仓库格数。调大后续轮次更能囤机，调小容量成长更慢；不增加单舰装备槽。</x:v>
       </x:c>
       <x:c r="F12" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -745,7 +745,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="48" customHeight="1">
+    <x:row r="13" ht="62" customHeight="1">
       <x:c r="A13" s="19" t="str">
         <x:v>initial_retention_capacity</x:v>
       </x:c>
@@ -756,10 +756,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D13" s="19" t="str">
-        <x:v>格</x:v>
+        <x:v>架</x:v>
       </x:c>
       <x:c r="E13" s="19" t="str">
-        <x:v>初始保留容量</x:v>
+        <x:v>保留名额初始基数，默认0；实际选择本次保留时加入累计增长及即将重铸的一次增长。调大名额更多，调小更少；不是首轮只能保留0架。</x:v>
       </x:c>
       <x:c r="F13" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -779,10 +779,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D14" s="19" t="str">
-        <x:v>格/重铸</x:v>
+        <x:v>架/次重铸</x:v>
       </x:c>
       <x:c r="E14" s="19" t="str">
-        <x:v>每次重铸增加保留格数</x:v>
+        <x:v>每次重铸增加保留名额，默认10，选择本次保留时计入即将重铸的一次。调大后续保留更多，调小更少；保留机封存到对应星球阶段开放，不保留材料。</x:v>
       </x:c>
       <x:c r="F14" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -791,7 +791,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="22" customHeight="1">
+    <x:row r="15" ht="48" customHeight="1">
       <x:c r="A15" s="19" t="str">
         <x:v>maximum_equipped</x:v>
       </x:c>
@@ -805,7 +805,7 @@
         <x:v>架</x:v>
       </x:c>
       <x:c r="E15" s="19" t="str">
-        <x:v>全局无人机装备上限</x:v>
+        <x:v>默认5。全局装备数量硬上限，范围1..5。调小限制同时生效架数；最终还受当前舰型容量限制，调大不能超过5。</x:v>
       </x:c>
       <x:c r="F15" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；1..5，硬上限5</x:v>
@@ -814,7 +814,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="22" customHeight="1">
+    <x:row r="16" ht="48" customHeight="1">
       <x:c r="A16" s="19" t="str">
         <x:v>maximum_legendary</x:v>
       </x:c>
@@ -828,7 +828,7 @@
         <x:v>架</x:v>
       </x:c>
       <x:c r="E16" s="19" t="str">
-        <x:v>同时装备传说数量上限</x:v>
+        <x:v>默认2。同时装备传说无人机上限，范围1..2。调小限制传说效果组合，调大允许更多组合但不能超过2；不是抽中传说的概率。</x:v>
       </x:c>
       <x:c r="F16" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；1..2，硬上限2</x:v>
@@ -837,7 +837,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="22" customHeight="1">
+    <x:row r="17" ht="48" customHeight="1">
       <x:c r="A17" s="19" t="str">
         <x:v>maximum_ultimate</x:v>
       </x:c>
@@ -851,7 +851,7 @@
         <x:v>架</x:v>
       </x:c>
       <x:c r="E17" s="19" t="str">
-        <x:v>同时装备究极数量上限</x:v>
+        <x:v>默认1。同时装备究极上限，现有合法值只能1。硬上限1，不提供多究极玩法；不是核心抽取概率。</x:v>
       </x:c>
       <x:c r="F17" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；必须为1，硬上限1</x:v>
@@ -871,10 +871,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D18" s="19" t="str">
-        <x:v>次/advance</x:v>
+        <x:v>次/一次advance</x:v>
       </x:c>
       <x:c r="E18" s="19" t="str">
-        <x:v>单次advance最多结算数，性能保护而非奖励倍率</x:v>
+        <x:v>默认8。固定单次推进最多结算8轮的性能保护。只读；积压工作由后续调用继续处理，不是奖励倍率或探索次数上限。</x:v>
       </x:c>
       <x:c r="F18" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关</x:v>
@@ -883,7 +883,7 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="48" customHeight="1">
+    <x:row r="19" ht="62" customHeight="1">
       <x:c r="A19" s="19" t="str">
         <x:v>ultimate_weapon_bonus</x:v>
       </x:c>
@@ -897,7 +897,7 @@
         <x:v>武器有效等级增量</x:v>
       </x:c>
       <x:c r="E19" s="19" t="str">
-        <x:v>究极武器等级增量覆盖普通来源加成，不叠加；究极状态优先</x:v>
+        <x:v>默认5。究极武器有效等级增量，覆盖普通/蓝来源/传说等级加成而不叠加。调大究极输出通常更强，调小更弱；不提高实际购买等级或改造费用。</x:v>
       </x:c>
       <x:c r="F19" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -917,10 +917,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D20" s="19" t="str">
-        <x:v>无量纲/按字段</x:v>
+        <x:v>概率，0..1</x:v>
       </x:c>
       <x:c r="E20" s="19" t="str">
-        <x:v>首个潜在槽成功概率；潜在槽失败不停止后续抽取</x:v>
+        <x:v>默认1。首个潜在词缀槽生成成功概率。调大更易生成词缀，调小更少；后续槽乘追加因子，某槽失败不停止后续抽取。限制0..1。</x:v>
       </x:c>
       <x:c r="F20" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；0≤value≤1</x:v>
@@ -940,10 +940,10 @@
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="D21" s="19" t="str">
-        <x:v>无量纲/按字段</x:v>
+        <x:v>概率，0..1</x:v>
       </x:c>
       <x:c r="E21" s="19" t="str">
-        <x:v>首个潜在槽成功概率；潜在槽失败不停止后续抽取</x:v>
+        <x:v>默认0.2。首个潜在挂设槽生成成功概率。调大更易带挂设，调小更少；后续槽乘追加因子，某槽失败不停止后续抽取。限制0..1。</x:v>
       </x:c>
       <x:c r="F21" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；0≤value≤1</x:v>
@@ -952,7 +952,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="48" customHeight="1">
+    <x:row r="22" ht="62" customHeight="1">
       <x:c r="A22" s="19" t="str">
         <x:v>additional_probability_factor</x:v>
       </x:c>
@@ -963,10 +963,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="D22" s="19" t="str">
-        <x:v>无量纲/按字段</x:v>
+        <x:v>概率递乘因子，0..1</x:v>
       </x:c>
       <x:c r="E22" s="19" t="str">
-        <x:v>后续潜在槽概率乘数；不因前槽失败提前停止抽取</x:v>
+        <x:v>默认0.25。潜在槽每向后一个位置，概率再乘此因子。调大后续槽更易成功，调小更稀少。例如起始0.2、因子0.25，前两槽概率0.2与0.05；失败不提前停止。</x:v>
       </x:c>
       <x:c r="F22" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；0≤value≤1</x:v>
@@ -975,7 +975,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="48" customHeight="1">
+    <x:row r="23" ht="62" customHeight="1">
       <x:c r="A23" s="19" t="str">
         <x:v>value_precision</x:v>
       </x:c>
@@ -986,10 +986,10 @@
         <x:v>0.001</x:v>
       </x:c>
       <x:c r="D23" s="19" t="str">
-        <x:v>无量纲/按字段</x:v>
+        <x:v>原始参数量化步长</x:v>
       </x:c>
       <x:c r="E23" s="19" t="str">
-        <x:v>随机参数量化网格</x:v>
+        <x:v>默认0.001。词缀及传说参数随机值的量化步长。调小候选值更细、保底MAX期望报价通常更高；调大值更粗。必须正数，各区间至少含一个量化点。</x:v>
       </x:c>
       <x:c r="F23" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；&gt;0</x:v>
@@ -998,7 +998,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="48" customHeight="1">
+    <x:row r="24" ht="62" customHeight="1">
       <x:c r="A24" s="19" t="str">
         <x:v>amplification_rate</x:v>
       </x:c>
@@ -1012,7 +1012,7 @@
         <x:v>每无人机等级复合增长率</x:v>
       </x:c>
       <x:c r="E24" s="19" t="str">
-        <x:v>每等级复合因子1+rate；0.05表示1.05</x:v>
+        <x:v>默认0.05。标记amplified的词缀按(1+此值)^(无人机等级−起点)放大。调大高于起点时更强、低于起点时缩小更多。例如0.05每级因子1.05；不是每级固定加5个百分点。</x:v>
       </x:c>
       <x:c r="F24" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -1035,7 +1035,7 @@
         <x:v>无人机等级</x:v>
       </x:c>
       <x:c r="E25" s="19" t="str">
-        <x:v>词缀复合放大指数起点，拟接线；当前冻结代码固定4。无人机level=start时原值×1，低于起点负指数缩小</x:v>
+        <x:v>默认4。词缀放大指数的零点，正式接线后生效。调大同等级词缀的放大值更小，调小更大；level=起点时×1，低于起点仍按负指数缩小。默认4与旧固定值等效。</x:v>
       </x:c>
       <x:c r="F25" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -1055,10 +1055,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D26" s="19" t="str">
-        <x:v>份</x:v>
+        <x:v>专属材料份/成功探索</x:v>
       </x:c>
       <x:c r="E26" s="19" t="str">
-        <x:v>探索基础材料奖励</x:v>
+        <x:v>默认1。探索基础专属材料奖励。调大各关奖励整体增加，调小减少；基础再加floor(max(0,关卡−成长起点)/步长)，最后乘补给倍率并向下取整。</x:v>
       </x:c>
       <x:c r="F26" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -1078,10 +1078,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D27" s="19" t="str">
-        <x:v>关/份</x:v>
+        <x:v>无人机/探索等级增量每份</x:v>
       </x:c>
       <x:c r="E27" s="19" t="str">
-        <x:v>每隔多少关增加1份基础材料</x:v>
+        <x:v>默认3。每隔多少探索关增加1份基础专属材料。调小成长更快，调大更慢；正整数。例如起点5、步长3，8关首次增加1份。</x:v>
       </x:c>
       <x:c r="F27" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -1101,10 +1101,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="D28" s="19" t="str">
-        <x:v>关</x:v>
+        <x:v>探索等级起点</x:v>
       </x:c>
       <x:c r="E28" s="19" t="str">
-        <x:v>材料成长起点，同时用于现代化报价；保留联动</x:v>
+        <x:v>默认5。材料奖励成长起点，同时是现代化费用等级项的原点。调大同关材料成长更晚且现代化等级项更低，调小反之；此联动保留，不拆成第二个价格起点。</x:v>
       </x:c>
       <x:c r="F28" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；奖励起点与改造价格既有联动不拆分</x:v>
@@ -1113,7 +1113,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="22" customHeight="1">
+    <x:row r="29" ht="48" customHeight="1">
       <x:c r="A29" s="19" t="str">
         <x:v>maximum_filter_conditions</x:v>
       </x:c>
@@ -1127,7 +1127,7 @@
         <x:v>条</x:v>
       </x:c>
       <x:c r="E29" s="19" t="str">
-        <x:v>筛选条件数量安全上限</x:v>
+        <x:v>默认5。固定筛选安全上限5条。只读；限制玩家规则复杂度，不调整无人机质量或奖励，不是筛选结果数量。</x:v>
       </x:c>
       <x:c r="F29" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；1..5，硬上限5</x:v>
@@ -1150,7 +1150,7 @@
         <x:v>字符</x:v>
       </x:c>
       <x:c r="E30" s="19" t="str">
-        <x:v>筛选导入文本长度安全上限</x:v>
+        <x:v>默认4096。固定筛选导入文本安全长度4096。只读；用于拒绝过大输入，不决定伤害、掉落或筛选概率。</x:v>
       </x:c>
       <x:c r="F30" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关</x:v>
@@ -1173,7 +1173,7 @@
         <x:v>次</x:v>
       </x:c>
       <x:c r="E31" s="19" t="str">
-        <x:v>改造预估循环次数安全上限</x:v>
+        <x:v>默认10000。固定改造保底预估循环保护10000次。只读；超过即报告预估限制，不能作为更高掉率或无限保底开关。</x:v>
       </x:c>
       <x:c r="F31" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关</x:v>
@@ -1182,7 +1182,7 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="48" customHeight="1">
+    <x:row r="32" ht="62" customHeight="1">
       <x:c r="A32" s="19" t="str">
         <x:v>lock_cost_multiplier</x:v>
       </x:c>
@@ -1193,10 +1193,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D32" s="19" t="str">
-        <x:v>无量纲/按字段</x:v>
+        <x:v>每个已锁词缀的费用倍率</x:v>
       </x:c>
       <x:c r="E32" s="19" t="str">
-        <x:v>每个已锁词缀对下次锁定费用的倍增系数</x:v>
+        <x:v>默认4。锁定费用=基础胶子费×此值^已锁词缀数。调大后续锁定更贵，调小更便宜；首次未锁时指数0。例如4时每增加一个已锁词缀，下一次费用再×4。</x:v>
       </x:c>
       <x:c r="F32" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -1205,7 +1205,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="48" customHeight="1">
+    <x:row r="33" ht="62" customHeight="1">
       <x:c r="A33" s="19" t="str">
         <x:v>reroll_guarantee_multiplier</x:v>
       </x:c>
@@ -1216,10 +1216,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D33" s="19" t="str">
-        <x:v>无量纲/按字段</x:v>
+        <x:v>期望成本乘数</x:v>
       </x:c>
       <x:c r="E33" s="19" t="str">
-        <x:v>保底最大值重洗的期望价倍数</x:v>
+        <x:v>默认3。保底MAX重洗报价=基础反质子费×各重洗区间可取值数量乘积×此值，并向上取整。调大保底更贵，调小更便宜；不改变MAX结果或普通随机重洗范围。</x:v>
       </x:c>
       <x:c r="F33" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -1228,7 +1228,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="48" customHeight="1">
+    <x:row r="34" ht="62" customHeight="1">
       <x:c r="A34" s="19" t="str">
         <x:v>modernization_cost_base</x:v>
       </x:c>
@@ -1239,10 +1239,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D34" s="19" t="str">
-        <x:v>材料份</x:v>
+        <x:v>材料份；也是舍入粒度</x:v>
       </x:c>
       <x:c r="E34" s="19" t="str">
-        <x:v>现代化费用基数与舍入粒度</x:v>
+        <x:v>默认10。现代化价格公式的材料基数，也是最终报价舍入粒度。调大通常更贵且报价更粗，调小更便宜且更细；价格按round(原价/此值)×此值，不改实际提升目标。</x:v>
       </x:c>
       <x:c r="F34" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；&gt;0</x:v>
@@ -1262,10 +1262,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D35" s="19" t="str">
-        <x:v>关</x:v>
+        <x:v>探索/无人机等级增量</x:v>
       </x:c>
       <x:c r="E35" s="19" t="str">
-        <x:v>现代化等级成本步长</x:v>
+        <x:v>默认3。现代化费用等级项分母：(1+(目标关−材料成长起点)/此值)。调大等级费用增长更慢，调小更快；目标由该路线已有最佳记录决定，正数。</x:v>
       </x:c>
       <x:c r="F35" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；&gt;0；奖励起点与改造价格既有联动不拆分</x:v>
@@ -1285,10 +1285,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="D36" s="19" t="str">
-        <x:v>无量纲/按字段</x:v>
+        <x:v>费用倍率</x:v>
       </x:c>
       <x:c r="E36" s="19" t="str">
-        <x:v>传说现代化费用乘数</x:v>
+        <x:v>默认2。仅传说无人机现代化价格乘此值。调大传说升级更贵，调小更便宜；普通无人机不乘此倍率。例如2表示传说同条件费用×2。</x:v>
       </x:c>
       <x:c r="F36" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -1308,10 +1308,10 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="D37" s="19" t="str">
-        <x:v>关</x:v>
+        <x:v>已清主线关ID</x:v>
       </x:c>
       <x:c r="E37" s="19" t="str">
-        <x:v>已通主线关卡达到后期补给门槛</x:v>
+        <x:v>默认60。后期补给门槛，须该主线关已通关，而不是仅最高到达。调大更晚开始补给，调小更早；之后按在线爬升时长渐进，默认60。</x:v>
       </x:c>
       <x:c r="F37" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -1331,10 +1331,10 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D38" s="19" t="str">
-        <x:v>无量纲/按字段</x:v>
+        <x:v>基础速率的终值倍率</x:v>
       </x:c>
       <x:c r="E38" s="19" t="str">
-        <x:v>后期充能最大倍率</x:v>
+        <x:v>默认30。后期补给爬升终点的充能倍率。调大最终充能更快，调小更慢；从×1线性爬升到此倍率，另乘挂设效果，不是储能容量倍率。</x:v>
       </x:c>
       <x:c r="F38" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -1354,10 +1354,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D39" s="19" t="str">
-        <x:v>无量纲/按字段</x:v>
+        <x:v>专属材料终值倍率</x:v>
       </x:c>
       <x:c r="E39" s="19" t="str">
-        <x:v>后期材料最大倍率</x:v>
+        <x:v>默认4。后期补给爬升终点的专属材料奖励倍率。调大材料更多，调小更少；从×1线性爬升，结算份数向下取整。例如终点4即基础奖励×4。</x:v>
       </x:c>
       <x:c r="F39" s="19" t="str">
         <x:v>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -1377,10 +1377,10 @@
         <x:v>600</x:v>
       </x:c>
       <x:c r="D40" s="19" t="str">
-        <x:v>游戏秒</x:v>
+        <x:v>在线游戏秒</x:v>
       </x:c>
       <x:c r="E40" s="19" t="str">
-        <x:v>后期补给在线爬升时长</x:v>
+        <x:v>默认600。补给从×1到目标倍率的爬升时间。调大完全生效更晚，调小更快；只在线累计，离线不补进度，默认600游戏秒。</x:v>
       </x:c>
       <x:c r="F40" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；&gt;0</x:v>
@@ -1389,7 +1389,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="34" customHeight="1">
+    <x:row r="41" ht="48" customHeight="1">
       <x:c r="A41" s="19" t="str">
         <x:v>modernization_base_coefficient</x:v>
       </x:c>
@@ -1400,10 +1400,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D41" s="19" t="str">
-        <x:v>无量纲</x:v>
+        <x:v>无量纲费用系数</x:v>
       </x:c>
       <x:c r="E41" s="19" t="str">
-        <x:v>现代化费用初始系数；随后逐个加词缀阶级权重</x:v>
+        <x:v>默认1。现代化阶级系数=此值+逐个词缀的阶级费用权重。调大价格更高，调小更低；还乘等级项及传说倍率，默认1与旧固定值等效。</x:v>
       </x:c>
       <x:c r="F41" s="19" t="str">
         <x:v>&gt;0且有限；默认1.0；保留原公式、舍入顺序和奖励起点联动</x:v>
@@ -1412,7 +1412,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="48" customHeight="1">
+    <x:row r="42" ht="62" customHeight="1">
       <x:c r="A42" s="19" t="str">
         <x:v>auto_duration_crew_base</x:v>
       </x:c>
@@ -1423,10 +1423,10 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="D42" s="19" t="str">
-        <x:v>船员等级基数</x:v>
+        <x:v>船员等级折算基数</x:v>
       </x:c>
       <x:c r="E42" s="19" t="str">
-        <x:v>自动探索耗时船员等级折算基数</x:v>
+        <x:v>默认100。自动耗时=max(最低耗时,最佳手动X1秒数×B/(B+船员等级))。同一正等级时调大耗时更长，调小更短；B=100、等级100时记录耗时减半。</x:v>
       </x:c>
       <x:c r="F42" s="19" t="str">
         <x:v>&gt;0且有限；默认100；公共函数返回max(minimum_duration,best_x1*B/(B+L))，结算与UI共用</x:v>
@@ -1435,7 +1435,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="34" customHeight="1">
+    <x:row r="43" ht="62" customHeight="1">
       <x:c r="A43" s="19" t="str">
         <x:v>auto_ticket_crew_base</x:v>
       </x:c>
@@ -1446,10 +1446,10 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D43" s="19" t="str">
-        <x:v>船员等级基数</x:v>
+        <x:v>船员等级折算基数</x:v>
       </x:c>
       <x:c r="E43" s="19" t="str">
-        <x:v>自动探索票耗船员等级折算基数</x:v>
+        <x:v>默认20。自动票耗=基础票耗×B/(B+船员等级)。同一正等级时调大消耗更多，调小更少；B=20、等级20时半票。只调自动，失败退实际已付票，结算和UI共用公式。</x:v>
       </x:c>
       <x:c r="F43" s="19" t="str">
         <x:v>&gt;0且有限；默认20；公共函数ticket*B/(B+L)，三个消费者共用，不改满容量派发门槛</x:v>
@@ -1503,7 +1503,7 @@
       <x:c r="A2" s="13" t="str">
         <x:v>传说定义外键
 单位：已有ID引用
-约束：必须存在于传说定义；保持当前引用，变更需跨表校验</x:v>
+约束：必须存在于传说定义；保持当前引用，变更需跨表校验；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="B2" s="13" t="str">
         <x:v>固定输出/随机选择顺序；物理行排序不改变它
@@ -1513,7 +1513,7 @@
       <x:c r="C2" s="13" t="str">
         <x:v>该效果已实现参数名
 单位：稳定ID
-约束：仅已有实现/已验ID；不自动新增功能；非空；主键作用域唯一</x:v>
+约束：仅已有实现/已验ID；不自动新增功能；非空；主键作用域唯一；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="D2" s="13" t="str">
         <x:v>新生成/重洗范围下端
@@ -1559,7 +1559,7 @@
         <x:v>string</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="34" customHeight="1">
+    <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="19" t="str">
         <x:v>higgs_cannon</x:v>
       </x:c>
@@ -1576,13 +1576,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="F4" s="19" t="str">
-        <x:v>加成比例；2=+200%，实际×3</x:v>
+        <x:v>伤害加成比例</x:v>
       </x:c>
       <x:c r="G4" s="19" t="str">
-        <x:v>加到1后作伤害倍率，不是直接倍率</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="34" customHeight="1">
+        <x:v>炮伤乘1+本值；2表示×3。调大更强；只改变伤害，不改变宽度。 本页区间用于新生成/重洗，不自动重抽已有存值。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="19" t="str">
         <x:v>higgs_cannon</x:v>
       </x:c>
@@ -1602,10 +1602,10 @@
         <x:v>射线宽度加成比例</x:v>
       </x:c>
       <x:c r="G5" s="19" t="str">
-        <x:v>宽度倍率=1+area_bonus；1表示宽度×2，不是任意面积倍数</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="34" customHeight="1">
+        <x:v>射线宽度乘1+本值；1表示宽度×2。调大命中区域更宽；不是面积平方倍率。 本页区间用于新生成/重洗，不自动重抽已有存值。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="19" t="str">
         <x:v>scatter_pulse</x:v>
       </x:c>
@@ -1622,13 +1622,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="F6" s="19" t="str">
-        <x:v>加成比例；2=+200%，实际×3</x:v>
+        <x:v>单目标伤害加成比例</x:v>
       </x:c>
       <x:c r="G6" s="19" t="str">
-        <x:v>加到1后作伤害倍率，不是直接倍率</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="34" customHeight="1">
+        <x:v>场上仅一个有效目标时激光乘1+本值；2表示×3。调大单体更强，多目标时不生效。 本页区间用于新生成/重洗，不自动重抽已有存值。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="62" customHeight="1">
       <x:c r="A7" s="19" t="str">
         <x:v>prism_tower</x:v>
       </x:c>
@@ -1645,13 +1645,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="F7" s="19" t="str">
-        <x:v>既有激光最大倍率的加法增量</x:v>
+        <x:v>激光最大倍率加法增量</x:v>
       </x:c>
       <x:c r="G7" s="19" t="str">
-        <x:v>加到既有最大倍率，不是独立总倍率</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="22" customHeight="1">
+        <x:v>对该棱镜塔源既有激光最大倍率加本值，调大蓄满倍率更高，不是全部激光再乘本值。 本页区间用于新生成/重洗，不自动重抽已有存值。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="62" customHeight="1">
       <x:c r="A8" s="19" t="str">
         <x:v>strange_matter</x:v>
       </x:c>
@@ -1671,10 +1671,10 @@
         <x:v>直接伤害倍率</x:v>
       </x:c>
       <x:c r="G8" s="19" t="str">
-        <x:v>1.3表示伤害×1.3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="34" customHeight="1">
+        <x:v>延迟奇异物质伤害=炮击原伤×本值，1.3表示×1.3。调大后续伤害更强，不改变概率。 本页区间用于新生成/重洗，不自动重抽已有存值。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="62" customHeight="1">
       <x:c r="A9" s="19" t="str">
         <x:v>laser_charge</x:v>
       </x:c>
@@ -1691,13 +1691,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="F9" s="19" t="str">
-        <x:v>加成比例；2=+200%，实际×3</x:v>
+        <x:v>激光额外伤害比例上限</x:v>
       </x:c>
       <x:c r="G9" s="19" t="str">
-        <x:v>加到1后作伤害倍率，不是直接倍率</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="22" customHeight="1">
+        <x:v>额外比例取min(本值,每激光加成×激光来源数)，最终乘1+比例。调大只放宽上限，来源不足时不增伤。 本页区间用于新生成/重洗，不自动重抽已有存值。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="48" customHeight="1">
       <x:c r="A10" s="19" t="str">
         <x:v>wild_missile</x:v>
       </x:c>
@@ -1717,10 +1717,10 @@
         <x:v>直接伤害倍率</x:v>
       </x:c>
       <x:c r="G10" s="19" t="str">
-        <x:v>1.3表示伤害×1.3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="34" customHeight="1">
+        <x:v>特殊主导弹伤害乘本值，7表示×7。调大单次更强；触发间隔由attack_period另管。 本页区间用于新生成/重洗，不自动重抽已有存值。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="62" customHeight="1">
       <x:c r="A11" s="19" t="str">
         <x:v>endless_beam</x:v>
       </x:c>
@@ -1737,13 +1737,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="F11" s="19" t="str">
-        <x:v>既有激光最大倍率的加法增量</x:v>
+        <x:v>激光最大倍率加法增量</x:v>
       </x:c>
       <x:c r="G11" s="19" t="str">
-        <x:v>加到既有最大倍率，不是独立总倍率</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="34" customHeight="1">
+        <x:v>仅选定最强持续长激光源的既有最大倍率加本值。调大持续源更强，不同时新增多个持续源。 本页区间用于新生成/重洗，不自动重抽已有存值。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="62" customHeight="1">
       <x:c r="A12" s="19" t="str">
         <x:v>dodge_counter</x:v>
       </x:c>
@@ -1763,10 +1763,10 @@
         <x:v>闪避概率上限，0..1</x:v>
       </x:c>
       <x:c r="G12" s="19" t="str">
-        <x:v>实际闪避概率=min(现有武器最高暴击概率,上限)，不是固定实际闪避率</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="34" customHeight="1">
+        <x:v>实际概率=min(当前武器最高暴击概率,本值)。0.75为75%上限，不能保证实际75%；调大只解除上限限制。 本页区间用于新生成/重洗，不自动重抽已有存值。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="48" customHeight="1">
       <x:c r="A13" s="19" t="str">
         <x:v>dodge_counter</x:v>
       </x:c>
@@ -1783,13 +1783,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F13" s="19" t="str">
-        <x:v>加成比例；2=+200%，实际×3</x:v>
+        <x:v>反击伤害加成比例</x:v>
       </x:c>
       <x:c r="G13" s="19" t="str">
-        <x:v>加到1后作伤害倍率，不是直接倍率</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="34" customHeight="1">
+        <x:v>反击随机现有武器伤害乘1+本值，0.7表示×1.7。调大反击更强，不提高闪避概率。 本页区间用于新生成/重洗，不自动重抽已有存值。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="62" customHeight="1">
       <x:c r="A14" s="19" t="str">
         <x:v>drone_master</x:v>
       </x:c>
@@ -1806,13 +1806,13 @@
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="F14" s="19" t="str">
-        <x:v>上限减伤比例</x:v>
+        <x:v>减伤比例上限，0..1</x:v>
       </x:c>
       <x:c r="G14" s="19" t="str">
-        <x:v>按装备未失效无人机的最大品质系数/ultimate系数折算，取最大不累加；0.5是上限50%</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="22" customHeight="1">
+        <x:v>实际减伤=本值×未失效已装备机最大品质系数/究极系数。0.5为最高品质50%；品质系数取最大不加总。 本页区间用于新生成/重洗，不自动重抽已有存值。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="62" customHeight="1">
       <x:c r="A15" s="19" t="str">
         <x:v>black_hole</x:v>
       </x:c>
@@ -1829,13 +1829,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="F15" s="19" t="str">
-        <x:v>直接伤害倍率</x:v>
+        <x:v>释放伤害直接倍率</x:v>
       </x:c>
       <x:c r="G15" s="19" t="str">
-        <x:v>1.3表示伤害×1.3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="34" customHeight="1">
+        <x:v>黑洞释放伤害=吸收的己方原伤累计×本值。1.3表示×1.3；敌方伤害吸收用于防护，不计入释放伤害。 本页区间用于新生成/重洗，不自动重抽已有存值。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="62" customHeight="1">
       <x:c r="A16" s="19" t="str">
         <x:v>drone_rebuild</x:v>
       </x:c>
@@ -1852,10 +1852,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F16" s="19" t="str">
-        <x:v>每牺牲层伤害/防御加成比例</x:v>
+        <x:v>每牺牲一次的伤害/防御加成比例</x:v>
       </x:c>
       <x:c r="G16" s="19" t="str">
-        <x:v>逐次牺牲累加；0.7为每层+70%</x:v>
+        <x:v>每次重建牺牲一架可用无人机，累计加本值。0.7、两层累计+140%；调大每层更强，层上限另管。 本页区间用于新生成/重洗，不自动重抽已有存值。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1907,12 +1907,12 @@
       <x:c r="A2" s="13" t="str">
         <x:v>传说定义外键
 单位：已有ID引用
-约束：必须存在于传说定义；保持当前引用，变更需跨表校验</x:v>
+约束：必须存在于传说定义；保持当前引用，变更需跨表校验；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="B2" s="13" t="str">
         <x:v>效果内固定常量路径，如quality_ratios/white
 单位：相对字段路径
-约束：仅当前支持的已知路径，不接受脚本/任意表达式</x:v>
+约束：仅当前支持的已知路径，不接受脚本/任意表达式；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="C2" s="13" t="str">
         <x:v>本键固定数据类型，不随单元格显示格式改变
@@ -1985,10 +1985,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E4" s="19" t="str">
-        <x:v>炮类武器来源数上限/个</x:v>
+        <x:v>炮类武器来源数</x:v>
       </x:c>
       <x:c r="F4" s="19" t="str">
-        <x:v>higgs_cannon：maximum_cannon_sources；参与统计的炮类来源数上限；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>装备希格斯时允许的炮类武器来源总数上限，默认1；包含普通武器与无人机来源。调大允许更多炮来源，不提高每炮伤害。</x:v>
       </x:c>
       <x:c r="G4" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -1997,7 +1997,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="62" customHeight="1">
+    <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="19" t="str">
         <x:v>precise_guidance</x:v>
       </x:c>
@@ -2014,7 +2014,7 @@
         <x:v>每已有层数的复合倍率底数</x:v>
       </x:c>
       <x:c r="F5" s="19" t="str">
-        <x:v>precise_guidance：stack_multiplier；伤害=base×multiplier^layers，不是每层相加；limit关闭时stack_limit不参与；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>伤害乘B^目标已有层数；B=1.5时2层×2.25。调大成长更快。每主发射批次每目标只叠一次，不按导弹颗数。</x:v>
       </x:c>
       <x:c r="G5" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -2040,7 +2040,7 @@
         <x:v>开关</x:v>
       </x:c>
       <x:c r="F6" s="19" t="str">
-        <x:v>precise_guidance：stack_limit_enabled；关闭时stack_limit不参与；不是倍率；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>是否启用叠层上限。false时stack_limit完全不参与；true限制后续累计层数。默认关闭，开启不改变单发记层方式。</x:v>
       </x:c>
       <x:c r="G6" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -2066,7 +2066,7 @@
         <x:v>层</x:v>
       </x:c>
       <x:c r="F7" s="19" t="str">
-        <x:v>precise_guidance：stack_limit；堆叠层数；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>启用上限时最多保留的目标层数；调大允许更高复合伤害；0且启用会保持0层。默认0且关闭，不等于默认无制导。</x:v>
       </x:c>
       <x:c r="G7" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -2089,10 +2089,10 @@
         <x:v>first_hit_per_batch_per_target</x:v>
       </x:c>
       <x:c r="E8" s="19" t="str">
-        <x:v>无量纲/固定枚举</x:v>
+        <x:v>固定行为声明</x:v>
       </x:c>
       <x:c r="F8" s="19" t="str">
-        <x:v>precise_guidance：counting_policy；现有固定效果语义；不新增消费者；已实现传说效果参数区间与固定常量；当前行为是固定实现，不通过此字段改变</x:v>
+        <x:v>锁定：每发射批次每目标首次命中记一次。字段本身无消费者，改文字不改变逻辑。</x:v>
       </x:c>
       <x:c r="G8" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关</x:v>
@@ -2118,7 +2118,7 @@
         <x:v>额外连锁目标/跳数</x:v>
       </x:c>
       <x:c r="F9" s="19" t="str">
-        <x:v>prism_tower：nearby_targets；连锁额外目标数；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>棱镜塔连锁额外目标计数，默认5；调大可打更多邻近目标，不含最初主目标，不增加塔数量。</x:v>
       </x:c>
       <x:c r="G9" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -2141,10 +2141,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E10" s="19" t="str">
-        <x:v>无量纲/固定枚举</x:v>
+        <x:v>固定塔来源数</x:v>
       </x:c>
       <x:c r="F10" s="19" t="str">
-        <x:v>prism_tower：maximum_towers；现有固定效果语义；不新增消费者；已实现传说效果参数区间与固定常量；当前行为是固定实现，不通过此字段改变</x:v>
+        <x:v>锁定1；代码只允许一个有效棱镜塔，此字段未消费，不是可扩塔开关。</x:v>
       </x:c>
       <x:c r="G10" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关</x:v>
@@ -2167,10 +2167,10 @@
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="E11" s="19" t="str">
-        <x:v>非击杀炮击命中生成1个的概率，0..1</x:v>
+        <x:v>非击杀炮命中的生成概率，0..1</x:v>
       </x:c>
       <x:c r="F11" s="19" t="str">
-        <x:v>strange_matter：spawn_probability；击杀分支使用kill_spawns绕过此概率；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>非击杀炮击命中时，以本概率生成1份延迟奇异物质；0.4=40%。击杀时直接用kill_spawns，不抽此概率。</x:v>
       </x:c>
       <x:c r="G11" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；0..1</x:v>
@@ -2196,7 +2196,7 @@
         <x:v>游戏秒</x:v>
       </x:c>
       <x:c r="F12" s="19" t="str">
-        <x:v>strange_matter：delay；按游戏时间计时；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>奇异物质生成后到造成伤害的延迟，默认1。调大伤害更晚，不增加份数或倍率。</x:v>
       </x:c>
       <x:c r="G12" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；当前支持计时参数&gt;0，黑洞周期不得短于吸收窗口</x:v>
@@ -2219,10 +2219,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="E13" s="19" t="str">
-        <x:v>个</x:v>
+        <x:v>份/击杀炮击</x:v>
       </x:c>
       <x:c r="F13" s="19" t="str">
-        <x:v>strange_matter：kill_spawns；击杀后生成数量；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>炮击击杀时直接生成的奇异物质份数，默认2；调大更多延迟伤害。派生触发不能再触发其他效果。</x:v>
       </x:c>
       <x:c r="G13" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -2245,10 +2245,10 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="E14" s="19" t="str">
-        <x:v>每激光来源加成比例</x:v>
+        <x:v>每个激光来源的加成比例</x:v>
       </x:c>
       <x:c r="F14" s="19" t="str">
-        <x:v>laser_charge：bonus_per_laser；每个激光来源的加成比例；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>每激光来源提供本比例，最终受maximum_bonus限制。0.5、两来源是+100%（若未达上限）；调大更快达上限。</x:v>
       </x:c>
       <x:c r="G14" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -2271,10 +2271,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E15" s="19" t="str">
-        <x:v>特殊攻击前的普通主导弹攻击批次数</x:v>
+        <x:v>特殊攻击前的普通主导弹批次数</x:v>
       </x:c>
       <x:c r="F15" s="19" t="str">
-        <x:v>wild_missile：attack_period；N=3为普通、普通、普通、特殊，总周期4；不按导弹颗数计数；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>N=3为普通、普通、普通、特殊，周期N+1次；调大特殊更稀疏。按主发射批次，不按颗数或秒。</x:v>
       </x:c>
       <x:c r="G15" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -2297,10 +2297,10 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="E16" s="19" t="str">
-        <x:v>主击伤害比例</x:v>
+        <x:v>主击伤害比例，0..1</x:v>
       </x:c>
       <x:c r="F16" s="19" t="str">
-        <x:v>wild_missile：blast_fraction；0.5表示主击伤害的50%；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>特殊导弹爆炸额外伤害=主击原伤×本值，0.5是50%。调大爆炸更强，不改变主击倍率或周期。</x:v>
       </x:c>
       <x:c r="G16" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；0..1</x:v>
@@ -2326,7 +2326,7 @@
         <x:v>游戏秒</x:v>
       </x:c>
       <x:c r="F17" s="19" t="str">
-        <x:v>dodge_counter：cooldown；按游戏时间计时；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>闪避反击之间的冷却，默认2；调大反击更稀疏。冷却限制反击，不把闪避概率改成每两秒固定一次。</x:v>
       </x:c>
       <x:c r="G17" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；当前支持计时参数&gt;0，黑洞周期不得短于吸收窗口</x:v>
@@ -2335,7 +2335,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="62" customHeight="1">
+    <x:row r="18" ht="76" customHeight="1">
       <x:c r="A18" s="19" t="str">
         <x:v>drone_master</x:v>
       </x:c>
@@ -2352,7 +2352,7 @@
         <x:v>无量纲相对品质系数</x:v>
       </x:c>
       <x:c r="F18" s="19" t="str">
-        <x:v>drone_master：white；统御取已装备未失效无人机最大品质系数/ultimate系数；ultimate是正数归一分母，不是各品质独立减伤概率；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>统御取未失效已装备机最高系数/究极系数，再乘减伤上限；不是本品质独立概率。增大此品质系数提高对应减伤；究极是正分母，改变它也影响所有其他品质，统一同比缩放不改结果。</x:v>
       </x:c>
       <x:c r="G18" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -2361,7 +2361,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="62" customHeight="1">
+    <x:row r="19" ht="76" customHeight="1">
       <x:c r="A19" s="19" t="str">
         <x:v>drone_master</x:v>
       </x:c>
@@ -2378,7 +2378,7 @@
         <x:v>无量纲相对品质系数</x:v>
       </x:c>
       <x:c r="F19" s="19" t="str">
-        <x:v>drone_master：blue；统御取已装备未失效无人机最大品质系数/ultimate系数；ultimate是正数归一分母，不是各品质独立减伤概率；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>统御取未失效已装备机最高系数/究极系数，再乘减伤上限；不是本品质独立概率。增大此品质系数提高对应减伤；究极是正分母，改变它也影响所有其他品质，统一同比缩放不改结果。</x:v>
       </x:c>
       <x:c r="G19" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -2387,7 +2387,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="62" customHeight="1">
+    <x:row r="20" ht="76" customHeight="1">
       <x:c r="A20" s="19" t="str">
         <x:v>drone_master</x:v>
       </x:c>
@@ -2404,7 +2404,7 @@
         <x:v>无量纲相对品质系数</x:v>
       </x:c>
       <x:c r="F20" s="19" t="str">
-        <x:v>drone_master：gold；统御取已装备未失效无人机最大品质系数/ultimate系数；ultimate是正数归一分母，不是各品质独立减伤概率；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>统御取未失效已装备机最高系数/究极系数，再乘减伤上限；不是本品质独立概率。增大此品质系数提高对应减伤；究极是正分母，改变它也影响所有其他品质，统一同比缩放不改结果。</x:v>
       </x:c>
       <x:c r="G20" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -2413,7 +2413,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="62" customHeight="1">
+    <x:row r="21" ht="76" customHeight="1">
       <x:c r="A21" s="19" t="str">
         <x:v>drone_master</x:v>
       </x:c>
@@ -2430,7 +2430,7 @@
         <x:v>无量纲相对品质系数</x:v>
       </x:c>
       <x:c r="F21" s="19" t="str">
-        <x:v>drone_master：legendary；统御取已装备未失效无人机最大品质系数/ultimate系数；ultimate是正数归一分母，不是各品质独立减伤概率；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>统御取未失效已装备机最高系数/究极系数，再乘减伤上限；不是本品质独立概率。增大此品质系数提高对应减伤；究极是正分母，改变它也影响所有其他品质，统一同比缩放不改结果。</x:v>
       </x:c>
       <x:c r="G21" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -2439,7 +2439,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="62" customHeight="1">
+    <x:row r="22" ht="76" customHeight="1">
       <x:c r="A22" s="19" t="str">
         <x:v>drone_master</x:v>
       </x:c>
@@ -2456,7 +2456,7 @@
         <x:v>无量纲相对品质系数</x:v>
       </x:c>
       <x:c r="F22" s="19" t="str">
-        <x:v>drone_master：ultimate；统御取已装备未失效无人机最大品质系数/ultimate系数；ultimate是正数归一分母，不是各品质独立减伤概率；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>统御取未失效已装备机最高系数/究极系数，再乘减伤上限；不是本品质独立概率。增大此品质系数提高对应减伤；究极是正分母，改变它也影响所有其他品质，统一同比缩放不改结果。</x:v>
       </x:c>
       <x:c r="G22" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；&gt;0，作为统御归一化分母</x:v>
@@ -2482,7 +2482,7 @@
         <x:v>游戏秒</x:v>
       </x:c>
       <x:c r="F23" s="19" t="str">
-        <x:v>black_hole：period；按游戏时间计时；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>黑洞循环周期，从一次开启到下次开启；默认20含5秒吸收窗口。调大开启更稀疏；需≥吸收时长且&gt;0。</x:v>
       </x:c>
       <x:c r="G23" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；当前支持计时参数&gt;0，黑洞周期不得短于吸收窗口</x:v>
@@ -2508,7 +2508,7 @@
         <x:v>游戏秒</x:v>
       </x:c>
       <x:c r="F24" s="19" t="str">
-        <x:v>black_hole：absorption_duration；按游戏时间计时；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>每次黑洞吸收窗口，默认5。调大吸收更久并更晚释放累计伤害；不得超过period。</x:v>
       </x:c>
       <x:c r="G24" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；当前支持计时参数&gt;0，黑洞周期不得短于吸收窗口</x:v>
@@ -2531,10 +2531,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E25" s="19" t="str">
-        <x:v>层</x:v>
+        <x:v>层/一场战斗</x:v>
       </x:c>
       <x:c r="F25" s="19" t="str">
-        <x:v>drone_rebuild：maximum_stacks；堆叠层数；已实现传说效果参数区间与固定常量</x:v>
+        <x:v>重建最大累计牺牲/加成层数，默认4。调大最多牺牲更多，仍受当前可用无人机数量限制，战斗重置。</x:v>
       </x:c>
       <x:c r="G25" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
@@ -2576,7 +2576,7 @@
         <x:v>amount</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="124" customHeight="1">
+    <x:row r="2" ht="194" customHeight="1">
       <x:c r="A2" s="13" t="str">
         <x:v>已有改造操作输出顺序
 单位：0起序号
@@ -2585,12 +2585,12 @@
       <x:c r="B2" s="13" t="str">
         <x:v>已有Forge操作ID
 单位：稳定ID
-约束：仅已有实现/已验ID；不自动新增功能；非空；主键作用域唯一</x:v>
+约束：仅已有实现/已验ID；不自动新增功能；非空；主键作用域唯一；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="C2" s="13" t="str">
-        <x:v>现有材料或ultimate_cores
+        <x:v>费用资源结构引用；当前为固定身份，只读，不因显示editable就能换资源。
 单位：已有ID引用
-约束：必须存在于路线材料与核心账本；保持当前引用，变更需跨表校验</x:v>
+约束：必须存在于路线材料与核心账本；保持当前引用，变更需跨表校验；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="D2" s="13" t="str">
         <x:v>同一操作中资源键的原插入顺序
@@ -2598,7 +2598,7 @@
 约束：同operation内唯一连续且锁定，不能依物理行排序</x:v>
       </x:c>
       <x:c r="E2" s="13" t="str">
-        <x:v>该操作消耗该资源的基础数量
+        <x:v>指定操作每次基础资源消耗。调大更贵；锁定/定向/保底操作还叠加其倍率或抽取次数；究极还原消耗核心，不退款。
 单位：份/次
 约束：非负整数；同(operation,resource)唯一；真实preview/commit共用此来源</x:v>
       </x:c>
@@ -2627,7 +2627,7 @@
       <x:c r="B4" s="19" t="str">
         <x:v>add_affix</x:v>
       </x:c>
-      <x:c r="C4" s="20" t="str">
+      <x:c r="C4" s="19" t="str">
         <x:v>degenerate_matter</x:v>
       </x:c>
       <x:c r="D4" s="29" t="n">
@@ -2644,7 +2644,7 @@
       <x:c r="B5" s="19" t="str">
         <x:v>replace_affix</x:v>
       </x:c>
-      <x:c r="C5" s="20" t="str">
+      <x:c r="C5" s="19" t="str">
         <x:v>degenerate_matter</x:v>
       </x:c>
       <x:c r="D5" s="29" t="n">
@@ -2661,7 +2661,7 @@
       <x:c r="B6" s="19" t="str">
         <x:v>add_hanging_slot</x:v>
       </x:c>
-      <x:c r="C6" s="20" t="str">
+      <x:c r="C6" s="19" t="str">
         <x:v>glueball</x:v>
       </x:c>
       <x:c r="D6" s="29" t="n">
@@ -2678,7 +2678,7 @@
       <x:c r="B7" s="19" t="str">
         <x:v>lock_affix</x:v>
       </x:c>
-      <x:c r="C7" s="20" t="str">
+      <x:c r="C7" s="19" t="str">
         <x:v>glueball</x:v>
       </x:c>
       <x:c r="D7" s="29" t="n">
@@ -2695,7 +2695,7 @@
       <x:c r="B8" s="19" t="str">
         <x:v>promote_affix</x:v>
       </x:c>
-      <x:c r="C8" s="20" t="str">
+      <x:c r="C8" s="19" t="str">
         <x:v>antiproton</x:v>
       </x:c>
       <x:c r="D8" s="29" t="n">
@@ -2712,7 +2712,7 @@
       <x:c r="B9" s="19" t="str">
         <x:v>reroll_values</x:v>
       </x:c>
-      <x:c r="C9" s="20" t="str">
+      <x:c r="C9" s="19" t="str">
         <x:v>antiproton</x:v>
       </x:c>
       <x:c r="D9" s="29" t="n">
@@ -2729,7 +2729,7 @@
       <x:c r="B10" s="19" t="str">
         <x:v>enable_omen</x:v>
       </x:c>
-      <x:c r="C10" s="20" t="str">
+      <x:c r="C10" s="19" t="str">
         <x:v>zero_point_energy</x:v>
       </x:c>
       <x:c r="D10" s="29" t="n">
@@ -2746,7 +2746,7 @@
       <x:c r="B11" s="19" t="str">
         <x:v>legendary</x:v>
       </x:c>
-      <x:c r="C11" s="20" t="str">
+      <x:c r="C11" s="19" t="str">
         <x:v>zero_point_energy</x:v>
       </x:c>
       <x:c r="D11" s="29" t="n">
@@ -2763,7 +2763,7 @@
       <x:c r="B12" s="19" t="str">
         <x:v>ultimate</x:v>
       </x:c>
-      <x:c r="C12" s="20" t="str">
+      <x:c r="C12" s="19" t="str">
         <x:v>ultimate_cores</x:v>
       </x:c>
       <x:c r="D12" s="29" t="n">
@@ -2780,7 +2780,7 @@
       <x:c r="B13" s="19" t="str">
         <x:v>restore_ultimate</x:v>
       </x:c>
-      <x:c r="C13" s="20" t="str">
+      <x:c r="C13" s="19" t="str">
         <x:v>ultimate_cores</x:v>
       </x:c>
       <x:c r="D13" s="29" t="n">
@@ -2835,7 +2835,7 @@
       <x:c r="A2" s="13" t="str">
         <x:v>保护参数或已存在policies子键
 单位：稳定键
-约束：允许清单，路径映射由契约指定</x:v>
+约束：允许清单，路径映射由契约指定；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="B2" s="13" t="str">
         <x:v>本键固定数据类型，不随单元格显示格式改变
@@ -2948,10 +2948,10 @@
         <x:v>exclusive</x:v>
       </x:c>
       <x:c r="D6" s="19" t="str">
-        <x:v>枚举/null</x:v>
+        <x:v>固定奖励策略</x:v>
       </x:c>
       <x:c r="E6" s="19" t="str">
-        <x:v>已支持策略或固定规则声明；未消费项锁定</x:v>
+        <x:v>抽到究极核心结果时，只发1个核心，不同时生成无人机。固定规则，不调整核心数量或赠机。</x:v>
       </x:c>
       <x:c r="F6" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -2971,10 +2971,10 @@
         <x:v>weighted_draw_stronger</x:v>
       </x:c>
       <x:c r="D7" s="19" t="str">
-        <x:v>枚举/null</x:v>
+        <x:v>固定升阶策略</x:v>
       </x:c>
       <x:c r="E7" s="19" t="str">
-        <x:v>已支持策略或固定规则声明；未消费项锁定</x:v>
+        <x:v>按阶级权重抽签，抽到比当前更强的阶才成功；成功只提升1阶，不直接跳到抽中阶。固定规则。</x:v>
       </x:c>
       <x:c r="F7" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -2994,10 +2994,10 @@
         <x:v>drone</x:v>
       </x:c>
       <x:c r="D8" s="19" t="str">
-        <x:v>枚举/null</x:v>
+        <x:v>固定预兆作用域</x:v>
       </x:c>
       <x:c r="E8" s="19" t="str">
-        <x:v>已支持策略或固定规则声明；未消费项锁定</x:v>
+        <x:v>预兆作用于该架无人机，筛选该机可修改词缀中的最低阶目标；不跨无人机生效。固定规则。</x:v>
       </x:c>
       <x:c r="F8" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -3017,10 +3017,10 @@
         <x:v>strongest_primary_stable_id</x:v>
       </x:c>
       <x:c r="D9" s="19" t="str">
-        <x:v>枚举/null</x:v>
+        <x:v>未消费的旧声明</x:v>
       </x:c>
       <x:c r="E9" s="19" t="str">
-        <x:v>已支持策略或固定规则声明；未消费项锁定</x:v>
+        <x:v>旧声明不驱动当前传说效果抽取。实际先按武器筛选适用效果，再均匀随机抽取，不按此strongest字符串挑最强。装备聚合时的同效果强弱选择是另一固定消费者。只读。</x:v>
       </x:c>
       <x:c r="F9" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -3040,10 +3040,10 @@
         <x:v>reached_planet_stage</x:v>
       </x:c>
       <x:c r="D10" s="19" t="str">
-        <x:v>枚举/null</x:v>
+        <x:v>固定封存领取声明</x:v>
       </x:c>
       <x:c r="E10" s="19" t="str">
-        <x:v>已支持策略或固定规则声明；未消费项锁定</x:v>
+        <x:v>重铸保留的无人机先封存，重新达到该机对应星球阶段后才能领取。实际门槛由正式星球数据和固定权限规则执行，此字符串本身不改变门槛。只读。</x:v>
       </x:c>
       <x:c r="F10" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -3061,10 +3061,10 @@
       </x:c>
       <x:c r="C11" s="19"/>
       <x:c r="D11" s="19" t="str">
-        <x:v>枚举/null</x:v>
+        <x:v>未接入预留项</x:v>
       </x:c>
       <x:c r="E11" s="19" t="str">
-        <x:v>已支持策略或固定规则声明；未消费项锁定</x:v>
+        <x:v>预留null，目前未接入消费，不提供重复传说动作开关；保持null，只读。</x:v>
       </x:c>
       <x:c r="F11" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -3084,10 +3084,10 @@
         <x:v>iron_income</x:v>
       </x:c>
       <x:c r="D12" s="19" t="str">
-        <x:v>效果标签</x:v>
+        <x:v>固定模块路由提示</x:v>
       </x:c>
       <x:c r="E12" s="19" t="str">
-        <x:v>已实现挂设的经验与效果成长；effects是声明，真实接入按固定模块ID分支，不读取这组字符串</x:v>
+        <x:v>资源采集器的铁收入效果提示。实际按固定resource_collector模块ID接入铁资源消费者，此字符串本身不改变效果。只读。</x:v>
       </x:c>
       <x:c r="F12" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -3107,10 +3107,10 @@
         <x:v>uranium_income</x:v>
       </x:c>
       <x:c r="D13" s="19" t="str">
-        <x:v>效果标签</x:v>
+        <x:v>固定模块路由提示</x:v>
       </x:c>
       <x:c r="E13" s="19" t="str">
-        <x:v>已实现挂设的经验与效果成长；effects是声明，真实接入按固定模块ID分支，不读取这组字符串</x:v>
+        <x:v>资源采集器的铀收入效果提示。实际按固定resource_collector模块ID接入铀资源消费者，此字符串本身不改变效果。只读。</x:v>
       </x:c>
       <x:c r="F13" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -3130,10 +3130,10 @@
         <x:v>ai_speed</x:v>
       </x:c>
       <x:c r="D14" s="19" t="str">
-        <x:v>效果标签</x:v>
+        <x:v>固定模块路由提示</x:v>
       </x:c>
       <x:c r="E14" s="19" t="str">
-        <x:v>已实现挂设的经验与效果成长；effects是声明，真实接入按固定模块ID分支，不读取这组字符串</x:v>
+        <x:v>分布式算法的AI效率效果提示。实际按固定distributed_algorithm模块ID接入AI研究效率，此字符串本身不改变效果。只读。</x:v>
       </x:c>
       <x:c r="F14" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -3153,10 +3153,10 @@
         <x:v>reactor_energy_cap</x:v>
       </x:c>
       <x:c r="D15" s="19" t="str">
-        <x:v>效果标签</x:v>
+        <x:v>固定模块路由提示</x:v>
       </x:c>
       <x:c r="E15" s="19" t="str">
-        <x:v>已实现挂设的经验与效果成长；effects是声明，真实接入按固定模块ID分支，不读取这组字符串</x:v>
+        <x:v>额外储能的反应炉能量容量效果提示。实际按固定extra_storage模块ID接入反应炉容量，此字符串本身不改变效果。只读。</x:v>
       </x:c>
       <x:c r="F15" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -3176,10 +3176,10 @@
         <x:v>gem_income</x:v>
       </x:c>
       <x:c r="D16" s="19" t="str">
-        <x:v>效果标签</x:v>
+        <x:v>固定模块路由提示</x:v>
       </x:c>
       <x:c r="E16" s="19" t="str">
-        <x:v>已实现挂设的经验与效果成长；effects是声明，真实接入按固定模块ID分支，不读取这组字符串</x:v>
+        <x:v>宝石精炼的强化碎片收益效果提示。实际按固定gem_refiner模块ID接入掉落及熔炼来源的强化碎片产出，此字符串本身不改变效果。只读。</x:v>
       </x:c>
       <x:c r="F16" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -3199,10 +3199,10 @@
         <x:v>hyperspace_energy_rate</x:v>
       </x:c>
       <x:c r="D17" s="19" t="str">
-        <x:v>效果标签</x:v>
+        <x:v>固定模块路由提示</x:v>
       </x:c>
       <x:c r="E17" s="19" t="str">
-        <x:v>已实现挂设的经验与效果成长；effects是声明，真实接入按固定模块ID分支，不读取这组字符串</x:v>
+        <x:v>异空间充能的能量充能速率效果提示。实际按固定hyperspace_charge模块ID接入在线充能，此字符串本身不改变效果。只读。</x:v>
       </x:c>
       <x:c r="F17" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -3222,10 +3222,10 @@
         <x:v>hyperspace_energy_cap</x:v>
       </x:c>
       <x:c r="D18" s="19" t="str">
-        <x:v>效果标签</x:v>
+        <x:v>固定模块路由提示</x:v>
       </x:c>
       <x:c r="E18" s="19" t="str">
-        <x:v>已实现挂设的经验与效果成长；effects是声明，真实接入按固定模块ID分支，不读取这组字符串</x:v>
+        <x:v>异空间充能的能量容量效果提示。实际按固定hyperspace_charge模块ID接入储能容量，此字符串本身不改变效果。只读。</x:v>
       </x:c>
       <x:c r="F18" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -3245,10 +3245,10 @@
         <x:v>0.8</x:v>
       </x:c>
       <x:c r="D19" s="19" t="str">
-        <x:v>倍率/比例/计数，见实体列定义</x:v>
+        <x:v>已有存值校验下界</x:v>
       </x:c>
       <x:c r="E19" s="19" t="str">
-        <x:v>已实现传说效果参数区间与固定常量；仅校验已有存值，不用于新抽取，旧档迁移不在本轮</x:v>
+        <x:v>仅用于验证已有统御maximum_reduction参数的兼容许可范围0.8..0.9；此项是下界0.8，不是新生成或重洗范围。只读，不做旧档迁移。</x:v>
       </x:c>
       <x:c r="F19" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -3268,10 +3268,10 @@
         <x:v>0.9</x:v>
       </x:c>
       <x:c r="D20" s="19" t="str">
-        <x:v>倍率/比例/计数，见实体列定义</x:v>
+        <x:v>已有存值校验上界</x:v>
       </x:c>
       <x:c r="E20" s="19" t="str">
-        <x:v>已实现传说效果参数区间与固定常量；仅校验已有存值，不用于新抽取，旧档迁移不在本轮</x:v>
+        <x:v>仅用于验证已有统御maximum_reduction参数的兼容许可范围0.8..0.9；此项是上界0.9，不是新生成或重洗范围。只读，不做旧档迁移。</x:v>
       </x:c>
       <x:c r="F20" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -3318,7 +3318,7 @@
       <x:c r="B2" s="13" t="str">
         <x:v>现有alpha/beta/gamma/delta路线
 单位：稳定ID
-约束：仅已有实现/已验ID；不自动新增功能；非空；主键作用域唯一</x:v>
+约束：仅已有实现/已验ID；不自动新增功能；非空；主键作用域唯一；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="C2" s="13" t="str">
         <x:v>路线武器结构绑定；四个既有ID唯一覆盖
@@ -3442,7 +3442,7 @@
         <x:v>dismantle_amount</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="152" customHeight="1">
+    <x:row r="2" ht="180" customHeight="1">
       <x:c r="A2" s="13" t="str">
         <x:v>固定输出/随机选择顺序；物理行排序不改变它
 单位：0起序号
@@ -3451,30 +3451,30 @@
       <x:c r="B2" s="13" t="str">
         <x:v>来源品质或独占核心抽签结果
 单位：稳定ID
-约束：white/blue/gold/legendary/ultimate_core固定集合；核心行的非weight列必须空</x:v>
+约束：white/blue/gold/legendary/ultimate_core固定集合；核心行的非weight列必须空；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="C2" s="13" t="str">
-        <x:v>结果相对抽签权重
+        <x:v>相对抽签权重，概率=本权重/所有结果总和；默认总和1.09。不是0.5独立50%。调大提高该结果相对出现率。
 单位：相对权重
 约束：非负；合计&gt;0；默认合计1.09，不能当互斥绝对概率</x:v>
       </x:c>
       <x:c r="D2" s="13" t="str">
-        <x:v>可生成/改造的词缀槽位上限
+        <x:v>词缀槽上限，受品质硬上限0/2/3/3；调大可生成/添加更多，不自动补已有机。
 单位：槽
 约束：非负；不超过既有0/2/3/3硬上限；仅ultimate_core行必须空，导出时不新增对应品质字段</x:v>
       </x:c>
       <x:c r="E2" s="13" t="str">
-        <x:v>可生成挂设槽位上限
+        <x:v>挂设槽上限，硬上限4/2/1/0；传说化保留原挂设，不能用传说0误解成清空。
 单位：槽
 约束：非负；不超过既有4/2/1/0硬上限；仅ultimate_core行必须空，导出时不新增对应品质字段</x:v>
       </x:c>
       <x:c r="F2" s="13" t="str">
-        <x:v>来源品质武器有效等级增量；非究极时蓝来源优先，蓝转传说仍用蓝加成
+        <x:v>非究极武器有效等级增量，蓝来源优先，蓝转传说继续用蓝值；究极覆盖，不叠加。
 单位：武器有效等级增量
 约束：非负；蓝来源继承规则不改；仅ultimate_core行必须空，导出时不新增对应品质字段</x:v>
       </x:c>
       <x:c r="G2" s="13" t="str">
-        <x:v>拆解专属材料数与随机挂设副本数
+        <x:v>一次拆解的专属材料份数及随机模块份数共用此值。首份模块解锁，重复增加经验；须与自动筛除奖励验证上限联动。
 单位：份/次
 约束：正整数；现行为同一个数，不拆成两个可独立调参来源；奖励校验上界联动；仅ultimate_core行必须空，导出时不新增对应品质字段</x:v>
       </x:c>
@@ -3643,10 +3643,10 @@
       <x:c r="B2" s="13" t="str">
         <x:v>现有舰型ID
 单位：已有ID引用
-约束：必须存在于ship.xlsx；保持当前引用，变更需跨表校验</x:v>
+约束：必须存在于ship.xlsx；保持当前引用，变更需跨表校验；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="C2" s="13" t="str">
-        <x:v>该舰型异空间无人机槽位
+        <x:v>该舰型无人机装备容量；调大可同时生效更多机，调小更少；仍受全局上限约束
 单位：架
 约束：1..5，且满足全局maximum_equipped</x:v>
       </x:c>
@@ -3746,7 +3746,7 @@
         <x:v>modernization_weight</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="138" customHeight="1">
+    <x:row r="2" ht="180" customHeight="1">
       <x:c r="A2" s="13" t="str">
         <x:v>固定输出/随机选择顺序；物理行排序不改变它
 单位：0起序号
@@ -3755,15 +3755,15 @@
       <x:c r="B2" s="13" t="str">
         <x:v>现有词缀阶级，1为最高
 单位：阶
-约束：1..5完整唯一</x:v>
+约束：1..5完整唯一；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="C2" s="13" t="str">
-        <x:v>生成/升阶判定使用的相对阶级权重
+        <x:v>生成及升阶成功判定相对权重；1阶最强。抽到更强阶即成功，但仅提升1阶，不跳阶。
 单位：相对权重
 约束：&gt;0；保留默认1/5/15/45/135及order</x:v>
       </x:c>
       <x:c r="D2" s="13" t="str">
-        <x:v>现代化费用附加阶级系数
+        <x:v>此阶每条普通词缀的现代化费用附加系数，与初始系数相加；调大该阶词缀越多报价越贵，不影响生成概率。
 单位：无量纲
 约束：非负；保留默认10/5/3/1/0.5；与draw_weight是不同用途，不混为一项</x:v>
       </x:c>
@@ -3890,7 +3890,7 @@
       <x:c r="B2" s="13" t="str">
         <x:v>已实现聚合器支持的词缀ID
 单位：稳定ID
-约束：仅已有实现/已验ID；不自动新增功能；非空；主键作用域唯一</x:v>
+约束：仅已有实现/已验ID；不自动新增功能；非空；主键作用域唯一；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="C2" s="13" t="str">
         <x:v>适用武器；空字符串代表全局
@@ -4110,24 +4110,24 @@
         <x:v>maximum</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="124" customHeight="1">
+    <x:row r="2" ht="194" customHeight="1">
       <x:c r="A2" s="13" t="str">
         <x:v>词缀定义外键
 单位：已有ID引用
-约束：必须存在于词缀定义；保持当前引用，变更需跨表校验</x:v>
+约束：必须存在于词缀定义；保持当前引用，变更需跨表校验；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="B2" s="13" t="str">
         <x:v>该词缀有定义的阶级
 单位：阶
-约束：1..5；仅导出存在的阶，不凭空补缺</x:v>
+约束：1..5；仅导出存在的阶，不凭空补缺；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="C2" s="13" t="str">
-        <x:v>未放大的原值区间下端
+        <x:v>原始词缀下界；比例词缀0.1=+10%，chain_count为数量。调大新抽取/重洗下限更高；未改已存值；区间含量化网格点。
 单位：原始加成；1=100%或数量
 约束：有限；≤maximum；value_precision网格至少有一个可取值</x:v>
       </x:c>
       <x:c r="D2" s="13" t="str">
-        <x:v>未放大的原值区间上端
+        <x:v>原始词缀上界，需≥下界；调大新抽取潜力更高，也会增加保底最大值期望成本；数量词缀最终聚合转int。
 单位：同minimum
 约束：有限；≥minimum；数量词缀现有量化及最终int投影保持</x:v>
       </x:c>
@@ -5055,7 +5055,7 @@
         <x:v>effects_note</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="138" customHeight="1">
+    <x:row r="2" ht="152" customHeight="1">
       <x:c r="A2" s="13" t="str">
         <x:v>固定输出/随机选择顺序；物理行排序不改变它
 单位：0起序号
@@ -5064,25 +5064,25 @@
       <x:c r="B2" s="13" t="str">
         <x:v>既有五种挂设ID
 单位：稳定ID
-约束：仅已有实现/已验ID；不自动新增功能；非空；主键作用域唯一</x:v>
+约束：仅已有实现/已验ID；不自动新增功能；非空；主键作用域唯一；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="C2" s="13" t="str">
-        <x:v>首份只解锁不给经验；重复模块输入经验及各级阈值共用base_exp
+        <x:v>每重复模块输入经验，同时各级阈值基数；首份只解锁。调大两者同比，不等于单纯更易升级。
 单位：经验/重复模块
 约束：&gt;0且有限</x:v>
       </x:c>
       <x:c r="D2" s="13" t="str">
-        <x:v>每级需求的增长率
+        <x:v>升级所需经验=base_exp×(1+本值)^当前等级。调大后续升级更慢。
 单位：比例；1=100%
 约束：≥0且有限，经验需求不得非有限</x:v>
       </x:c>
       <x:c r="E2" s="13" t="str">
-        <x:v>每架加成=(1+growth)^全局模块等级−1；等级0为0，同类多架相加
+        <x:v>每架已挂设加成=(1+本值)^全局模块等级−1。0.1、2级=21%，两架42%；仓库未装备不计。
 单位：比例；1=100%
 约束：≥0且有限，实际公式pow(1+g,L)-1保持</x:v>
       </x:c>
       <x:c r="F2" s="13" t="str">
-        <x:v>挂设可应用的最高到达关卡
+        <x:v>模块可挂设及参与效果的最高到达主线门槛；调大延后使用，不代表模块抽取概率。
 单位：关
 约束：非负整数</x:v>
       </x:c>
@@ -5268,7 +5268,7 @@
       <x:c r="B2" s="13" t="str">
         <x:v>既有十二种传说效果ID
 单位：稳定ID
-约束：仅已有实现/已验ID；不自动新增功能；非空；主键作用域唯一</x:v>
+约束：仅已有实现/已验ID；不自动新增功能；非空；主键作用域唯一；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
       </x:c>
       <x:c r="C2" s="13" t="str">
         <x:v>固定结构绑定；空字符串表示全武器通用

</xml_diff>

<commit_message>
Complete hyperspace visual configuration, drone appearance and forge guide; isolate omen replacement targeting
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/hyperspace_config.xlsx
+++ b/space-battleship/config_excel/hyperspace_config.xlsx
@@ -2,19 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础参数" sheetId="1" r:id="Rdbf188d28566469a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="路线" sheetId="2" r:id="R07cb589b63f848c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品质" sheetId="3" r:id="R0dd81bc0b9574ae7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="舰型容量" sheetId="4" r:id="R46bfb6ed1af5480e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶级权重" sheetId="5" r:id="R2c3c53182c2d429b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="词缀定义" sheetId="6" r:id="Rbea35f20e078402d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="词缀区间" sheetId="7" r:id="R6447d91b56bb48d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="挂设成长" sheetId="8" r:id="Rad73cc54c5e64ed1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="传说定义" sheetId="9" r:id="Rcc44ca8479a74b8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="传说随机参数" sheetId="10" r:id="R2a9f2c4c89cf47df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="传说常量" sheetId="11" r:id="R19ce7c85c67144c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改造费用" sheetId="12" r:id="Re49bd0df2c8b4b31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定规则_兼容说明" sheetId="13" r:id="Rac066a41c26f4176"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础参数" sheetId="1" r:id="R53127dd27fb84990"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="路线" sheetId="2" r:id="R54bba70b36c34e27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品质" sheetId="3" r:id="Rf1b9754b30594b15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="舰型容量" sheetId="4" r:id="R2c32f035015040fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶级权重" sheetId="5" r:id="R7e720a4f57324a0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="词缀定义" sheetId="6" r:id="R8101568e68984643"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="词缀区间" sheetId="7" r:id="Rb854cc478c954a9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="挂设成长" sheetId="8" r:id="R046d11685c9f4d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="传说定义" sheetId="9" r:id="R64310db33e234433"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="传说随机参数" sheetId="10" r:id="R82ba0e45b4b94956"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="传说常量" sheetId="11" r:id="R660f93728d044961"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改造费用" sheetId="12" r:id="R68b69f16cbd04721"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定规则_兼容说明" sheetId="13" r:id="R17db6601af48461a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="无人机外观" sheetId="14" r:id="R5c5bf9c6aade4646"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2997,7 +2998,7 @@
         <x:v>固定预兆作用域</x:v>
       </x:c>
       <x:c r="E8" s="19" t="str">
-        <x:v>预兆作用于该架无人机，筛选该机可修改词缀中的最低阶目标；不跨无人机生效。固定规则。</x:v>
+        <x:v>预兆仅在替换词缀时，优先选择该架未锁定词缀中的最低阶目标（T5先于T4，同阶随机）；不影响锁定或升阶，锁定从全部未锁词缀随机选择；不跨无人机生效。</x:v>
       </x:c>
       <x:c r="F8" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；现值锁定，只说明，不提供任意参数开关</x:v>
@@ -3278,6 +3279,475 @@
       </x:c>
       <x:c r="G20" s="23" t="b">
         <x:v>0</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="9" t="str">
+        <x:v>key</x:v>
+      </x:c>
+      <x:c r="B1" s="9" t="str">
+        <x:v>data_type</x:v>
+      </x:c>
+      <x:c r="C1" s="9" t="str">
+        <x:v>value</x:v>
+      </x:c>
+      <x:c r="D1" s="9" t="str">
+        <x:v>unit</x:v>
+      </x:c>
+      <x:c r="E1" s="9" t="str">
+        <x:v>description</x:v>
+      </x:c>
+      <x:c r="F1" s="9" t="str">
+        <x:v>constraint</x:v>
+      </x:c>
+      <x:c r="G1" s="9" t="str">
+        <x:v>editable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="124" customHeight="1">
+      <x:c r="A2" s="13" t="str">
+        <x:v>外观字段稳定路径，品质ID引用正式品质配置
+单位：稳定ID
+约束：仅已有实现/已验ID；不自动新增功能；非空；主键作用域唯一；固定结构身份列，必须与基线等值，不能只改物理行冒充结构变化</x:v>
+      </x:c>
+      <x:c r="B2" s="13" t="str">
+        <x:v>本键固定数据类型，不随单元格显示格式改变
+单位：类型标签
+约束：int/float/bool/string/null；必须符合键契约；锁定</x:v>
+      </x:c>
+      <x:c r="C2" s="13" t="str">
+        <x:v>按本键固定类型读入的单一字面值
+单位：见unit列
+约束：拒绝公式；固定字面类型；每字段范围/品质外键见本行constraint；有限值；不参与战斗数值</x:v>
+      </x:c>
+      <x:c r="D2" s="13" t="str">
+        <x:v>值的中文单位与比例口径
+单位：说明
+约束：必填；只作说明，不改变数值计算</x:v>
+      </x:c>
+      <x:c r="E2" s="13" t="str">
+        <x:v>逐字段中文用途、调大调小及纯表现边界
+单位：说明
+约束：必填；不参与JSON业务值</x:v>
+      </x:c>
+      <x:c r="F2" s="13" t="str">
+        <x:v>本字段固定类型、范围或品质外键限制
+单位：说明
+约束：必填；以代码契约执行，不能编辑此文案绕过校验</x:v>
+      </x:c>
+      <x:c r="G2" s="13" t="str">
+        <x:v>该键是否真实允许调整；不是功能开关
+单位：权限标签
+约束：锁定并匹配契约；false拒绝改离基线</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="20" customHeight="1">
+      <x:c r="A3" s="16" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="B3" s="16" t="str">
+        <x:v>enum</x:v>
+      </x:c>
+      <x:c r="C3" s="16" t="str">
+        <x:v>typed_literal</x:v>
+      </x:c>
+      <x:c r="D3" s="16" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="E3" s="16" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="F3" s="16" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="G3" s="16" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="48" customHeight="1">
+      <x:c r="A4" s="19" t="str">
+        <x:v>version</x:v>
+      </x:c>
+      <x:c r="B4" s="19" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="C4" s="24" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D4" s="19" t="str">
+        <x:v>缓存版本号</x:v>
+      </x:c>
+      <x:c r="E4" s="19" t="str">
+        <x:v>仅作表现缓存键，不代表数值或存档版本。调大或调小只改变缓存键；主场景_ready重读配置，内容变化清缓存，不逐帧读文件。</x:v>
+      </x:c>
+      <x:c r="F4" s="19" t="str">
+        <x:v>正整数</x:v>
+      </x:c>
+      <x:c r="G4" s="23" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="48" customHeight="1">
+      <x:c r="A5" s="19" t="str">
+        <x:v>quality.white.color</x:v>
+      </x:c>
+      <x:c r="B5" s="19" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="C5" s="20" t="str">
+        <x:v>b8c7d0</x:v>
+      </x:c>
+      <x:c r="D5" s="19" t="str">
+        <x:v>六位RGB十六进制</x:v>
+      </x:c>
+      <x:c r="E5" s="19" t="str">
+        <x:v>仓库和战场共用的白色品质标识色。更换色值改变标识色相；十六进制数值大小不代表品质强弱；白色机体保留模型原色。</x:v>
+      </x:c>
+      <x:c r="F5" s="19" t="str">
+        <x:v>六位hex；white须存在于正式品质配置</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="62" customHeight="1">
+      <x:c r="A6" s="19" t="str">
+        <x:v>quality.white.rank</x:v>
+      </x:c>
+      <x:c r="B6" s="19" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="C6" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="19" t="str">
+        <x:v>外侧结构档位</x:v>
+      </x:c>
+      <x:c r="E6" s="19" t="str">
+        <x:v>白色品质在仓库和战场共用的附加外侧结构档位。调大增加外侧结构，2起增加尾横条、3增加冠饰，调小减少结构；不改变抽取概率、属性或实际品质。</x:v>
+      </x:c>
+      <x:c r="F6" s="19" t="str">
+        <x:v>整数0..3；white须存在于正式品质配置</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="48" customHeight="1">
+      <x:c r="A7" s="19" t="str">
+        <x:v>quality.blue.color</x:v>
+      </x:c>
+      <x:c r="B7" s="19" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="C7" s="20" t="str">
+        <x:v>42c5ff</x:v>
+      </x:c>
+      <x:c r="D7" s="19" t="str">
+        <x:v>六位RGB十六进制</x:v>
+      </x:c>
+      <x:c r="E7" s="19" t="str">
+        <x:v>仓库和战场共用的蓝色品质标识色。更换色值改变色相；十六进制数值大小不代表品质强弱。</x:v>
+      </x:c>
+      <x:c r="F7" s="19" t="str">
+        <x:v>六位hex；blue须存在于正式品质配置</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="62" customHeight="1">
+      <x:c r="A8" s="19" t="str">
+        <x:v>quality.blue.rank</x:v>
+      </x:c>
+      <x:c r="B8" s="19" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="C8" s="24" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D8" s="19" t="str">
+        <x:v>外侧结构档位</x:v>
+      </x:c>
+      <x:c r="E8" s="19" t="str">
+        <x:v>蓝色品质在仓库和战场共用的附加外侧结构档位。调大增加外侧结构，2起增加尾横条、3增加冠饰，调小减少结构；不改变抽取概率、属性或实际品质。</x:v>
+      </x:c>
+      <x:c r="F8" s="19" t="str">
+        <x:v>整数0..3；blue须存在于正式品质配置</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="48" customHeight="1">
+      <x:c r="A9" s="19" t="str">
+        <x:v>quality.gold.color</x:v>
+      </x:c>
+      <x:c r="B9" s="19" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="C9" s="20" t="str">
+        <x:v>e5bb55</x:v>
+      </x:c>
+      <x:c r="D9" s="19" t="str">
+        <x:v>六位RGB十六进制</x:v>
+      </x:c>
+      <x:c r="E9" s="19" t="str">
+        <x:v>仓库和战场共用的金色品质标识色。更换色值改变色相；十六进制数值大小不代表品质强弱。</x:v>
+      </x:c>
+      <x:c r="F9" s="19" t="str">
+        <x:v>六位hex；gold须存在于正式品质配置</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="62" customHeight="1">
+      <x:c r="A10" s="19" t="str">
+        <x:v>quality.gold.rank</x:v>
+      </x:c>
+      <x:c r="B10" s="19" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="C10" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D10" s="19" t="str">
+        <x:v>外侧结构档位</x:v>
+      </x:c>
+      <x:c r="E10" s="19" t="str">
+        <x:v>金色品质在仓库和战场共用的附加外侧结构档位。调大增加外侧结构，2起增加尾横条、3增加冠饰，调小减少结构；不改变抽取概率、属性或实际品质。</x:v>
+      </x:c>
+      <x:c r="F10" s="19" t="str">
+        <x:v>整数0..3；gold须存在于正式品质配置</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="48" customHeight="1">
+      <x:c r="A11" s="19" t="str">
+        <x:v>quality.legendary.color</x:v>
+      </x:c>
+      <x:c r="B11" s="19" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="C11" s="20" t="str">
+        <x:v>bd83f4</x:v>
+      </x:c>
+      <x:c r="D11" s="19" t="str">
+        <x:v>六位RGB十六进制</x:v>
+      </x:c>
+      <x:c r="E11" s="19" t="str">
+        <x:v>仓库和战场共用的传说品质标识色。更换色值改变色相；十六进制数值大小不代表品质强弱。</x:v>
+      </x:c>
+      <x:c r="F11" s="19" t="str">
+        <x:v>六位hex；legendary须存在于正式品质配置</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="62" customHeight="1">
+      <x:c r="A12" s="19" t="str">
+        <x:v>quality.legendary.rank</x:v>
+      </x:c>
+      <x:c r="B12" s="19" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="C12" s="24" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D12" s="19" t="str">
+        <x:v>外侧结构档位</x:v>
+      </x:c>
+      <x:c r="E12" s="19" t="str">
+        <x:v>传说品质在仓库和战场共用的附加外侧结构档位。调大增加外侧结构，2起增加尾横条、3增加冠饰，调小减少结构；不改变抽取概率、属性或实际品质。</x:v>
+      </x:c>
+      <x:c r="F12" s="19" t="str">
+        <x:v>整数0..3；legendary须存在于正式品质配置</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="48" customHeight="1">
+      <x:c r="A13" s="19" t="str">
+        <x:v>ultimate_color</x:v>
+      </x:c>
+      <x:c r="B13" s="19" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="C13" s="20" t="str">
+        <x:v>7ef5e0</x:v>
+      </x:c>
+      <x:c r="D13" s="19" t="str">
+        <x:v>六位RGB十六进制</x:v>
+      </x:c>
+      <x:c r="E13" s="19" t="str">
+        <x:v>仓库和战场共用的究极状态视觉标识色（独立于品质）。更换色值改变色相；十六进制数值大小不代表品质强弱。</x:v>
+      </x:c>
+      <x:c r="F13" s="19" t="str">
+        <x:v>六位hex</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="19" t="str">
+        <x:v>emission</x:v>
+      </x:c>
+      <x:c r="B14" s="19" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="C14" s="24" t="n">
+        <x:v>0.28</x:v>
+      </x:c>
+      <x:c r="D14" s="19" t="str">
+        <x:v>自发光强度</x:v>
+      </x:c>
+      <x:c r="E14" s="19" t="str">
+        <x:v>仅战场3D饰件的发光强度。调大更亮，调小更暗；不改变仓库原始图标。</x:v>
+      </x:c>
+      <x:c r="F14" s="19" t="str">
+        <x:v>0..0.7</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="48" customHeight="1">
+      <x:c r="A15" s="19" t="str">
+        <x:v>animate</x:v>
+      </x:c>
+      <x:c r="B15" s="19" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+      <x:c r="C15" s="33" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D15" s="19" t="str">
+        <x:v>布尔开关</x:v>
+      </x:c>
+      <x:c r="E15" s="19" t="str">
+        <x:v>只控制究极装饰环随表现时钟旋转。true允许旋转，false停止旋转；QA冻结可覆盖。无数值大小比较，不改变战斗结算。</x:v>
+      </x:c>
+      <x:c r="F15" s="19" t="str">
+        <x:v>必须为bool</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="48" customHeight="1">
+      <x:c r="A16" s="19" t="str">
+        <x:v>high_tier_max</x:v>
+      </x:c>
+      <x:c r="B16" s="19" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="C16" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D16" s="19" t="str">
+        <x:v>阶级编号阈值</x:v>
+      </x:c>
+      <x:c r="E16" s="19" t="str">
+        <x:v>仓库和战场共用的高阶装饰最大阶级编号。T1最高，编号越小越稀有；调大覆盖更多阶级，调小仅保留更稀有阶级。</x:v>
+      </x:c>
+      <x:c r="F16" s="19" t="str">
+        <x:v>整数1..5</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="34" customHeight="1">
+      <x:c r="A17" s="19" t="str">
+        <x:v>ornament_scale</x:v>
+      </x:c>
+      <x:c r="B17" s="19" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="C17" s="24" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D17" s="19" t="str">
+        <x:v>装饰尺寸倍数</x:v>
+      </x:c>
+      <x:c r="E17" s="19" t="str">
+        <x:v>仅战场3D装饰相对尺寸。调大放大饰件，调小缩小饰件；不改变碰撞、属性或仓库图标。</x:v>
+      </x:c>
+      <x:c r="F17" s="19" t="str">
+        <x:v>0.5..1.1</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="62" customHeight="1">
+      <x:c r="A18" s="19" t="str">
+        <x:v>body_tint</x:v>
+      </x:c>
+      <x:c r="B18" s="19" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="C18" s="24" t="n">
+        <x:v>0.72</x:v>
+      </x:c>
+      <x:c r="D18" s="19" t="str">
+        <x:v>品质混色比例</x:v>
+      </x:c>
+      <x:c r="E18" s="19" t="str">
+        <x:v>仅战场3D中性装甲与品质色的混色比例。调大品质色更明显，调小更接近中性装甲；白色机体保留原色。仓库仍用原始图标、品质附加结构和色框。</x:v>
+      </x:c>
+      <x:c r="F18" s="19" t="str">
+        <x:v>0..1</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="34" customHeight="1">
+      <x:c r="A19" s="19" t="str">
+        <x:v>tier_glyph_scale</x:v>
+      </x:c>
+      <x:c r="B19" s="19" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="C19" s="24" t="n">
+        <x:v>2.8</x:v>
+      </x:c>
+      <x:c r="D19" s="19" t="str">
+        <x:v>阶级标识尺寸倍数</x:v>
+      </x:c>
+      <x:c r="E19" s="19" t="str">
+        <x:v>仅战场3D阶级几何标记尺寸。调大放大标识，调小缩小标识；不改变仓库原始图标。</x:v>
+      </x:c>
+      <x:c r="F19" s="19" t="str">
+        <x:v>1..3</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="b">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(config): scale hyperspace material units and rename collector
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/hyperspace_config.xlsx
+++ b/space-battleship/config_excel/hyperspace_config.xlsx
@@ -1459,6 +1459,52 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>material_unit_scale</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="C44" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>常规材料单位倍率</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>默认10。四种常规异空间材料的完整探索基础公式、拆解返还及改造消耗统一乘此倍率；究极核心数量和消耗不缩放。采集器另加产出倍率，最终取整；不能只改material_base_reward。</x:v>
+      </x:c>
+      <x:c r="F44" t="str">
+        <x:v>正整数，有限且&lt;9e15；究极核心除外；只作单位换算，不扩大无人机或挂设副本数量</x:v>
+      </x:c>
+      <x:c r="G44" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>ultimate_core_probability</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="C45" t="n">
+        <x:v>0.002</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>成功探索实际概率</x:v>
+      </x:c>
+      <x:c r="E45" t="str">
+        <x:v>默认0.002，即0.2%。究极核心独立实际掉落概率，不参与颜色品质权重归一化；不受幸运、材料单位倍率或采集器影响。quality_weights中旧ultimate_core项仅兼容，核心生成须忽略其权重。</x:v>
+      </x:c>
+      <x:c r="F45" t="str">
+        <x:v>有限概率，0≤value≤1；按实际概率抽样，不能作为相对品质权重</x:v>
+      </x:c>
+      <x:c r="G45" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3197,41 +3243,18 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="C17" s="19" t="str">
-        <x:v>hyperspace_energy_rate</x:v>
+        <x:v>hyperspace_material_income</x:v>
       </x:c>
       <x:c r="D17" s="19" t="str">
         <x:v>固定模块路由提示</x:v>
       </x:c>
       <x:c r="E17" s="19" t="str">
-        <x:v>异空间充能的能量充能速率效果提示。实际按固定hyperspace_charge模块ID接入在线充能，此字符串本身不改变效果。只读。</x:v>
+        <x:v>异空间采集器提升四种常规异空间材料产出，按(1+effect_growth)^模块等级，同类已装备加成相加，最终取整；究极核心除外。保留原模块ID和进度；此效果标识由固定契约注册。</x:v>
       </x:c>
       <x:c r="F17" s="19" t="str">
         <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关；现值锁定，只说明，不提供任意参数开关</x:v>
       </x:c>
       <x:c r="G17" s="23" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="76" customHeight="1">
-      <x:c r="A18" s="19" t="str">
-        <x:v>/hanging_modules/hyperspace_charge/effects/1</x:v>
-      </x:c>
-      <x:c r="B18" s="19" t="str">
-        <x:v>string</x:v>
-      </x:c>
-      <x:c r="C18" s="19" t="str">
-        <x:v>hyperspace_energy_cap</x:v>
-      </x:c>
-      <x:c r="D18" s="19" t="str">
-        <x:v>固定模块路由提示</x:v>
-      </x:c>
-      <x:c r="E18" s="19" t="str">
-        <x:v>异空间充能的能量容量效果提示。实际按固定hyperspace_charge模块ID接入储能容量，此字符串本身不改变效果。只读。</x:v>
-      </x:c>
-      <x:c r="F18" s="19" t="str">
-        <x:v>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；锁定，不提供任意玩法开关；现值锁定，只说明，不提供任意参数开关</x:v>
-      </x:c>
-      <x:c r="G18" s="23" t="b">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -5697,7 +5720,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="19" t="str">
-        <x:v>hyperspace_energy_rate；hyperspace_energy_cap</x:v>
+        <x:v>hyperspace_material_income</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Give equipped drones an independent body-level damage and capacity layer
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/hyperspace_config.xlsx
+++ b/space-battleship/config_excel/hyperspace_config.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="1" min="1" max="1"/>
@@ -1987,6 +1987,39 @@
         </is>
       </c>
       <c r="G45" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>drone_base_growth</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>每本体等级基础攻防倍率</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>默认1.05。每架装备无人机按此值^本体等级贡献额外倍率；多架额外部分相加，独立乘武器伤害和装甲/护盾上限。不依赖品质、词缀或挂载，不增加减伤。</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>有限数字，1≤值&lt;9e15；独立基础乘区；本体等级至少1</t>
+        </is>
+      </c>
+      <c r="G46" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Stage reactor automation and drone support candidates; pending gameplay and UI acceptance
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/hyperspace_config.xlsx
+++ b/space-battleship/config_excel/hyperspace_config.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="1" min="1" max="1"/>
@@ -1987,6 +1987,39 @@
         </is>
       </c>
       <c r="G45" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>drone_base_growth</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>每本体等级基础攻防倍率</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>默认1.05。每架装备无人机按此值^本体等级贡献额外倍率；多架额外部分相加，独立乘武器伤害和装甲/护盾上限。不依赖品质、词缀或挂载，不增加减伤。</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>有限数字，1≤值&lt;9e15；独立基础乘区；本体等级至少1</t>
+        </is>
+      </c>
+      <c r="G46" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: rebalance stages four to seven and add equipment evolution
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/hyperspace_config.xlsx
+++ b/space-battleship/config_excel/hyperspace_config.xlsx
@@ -539,24 +539,34 @@
         <x:v>bool</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="62" customHeight="1">
-      <x:c r="A4" s="19" t="str">
-        <x:v>unlock_stage</x:v>
-      </x:c>
-      <x:c r="B4" s="19" t="str">
-        <x:v>int</x:v>
+    <x:row r="4" ht="62" customHeight="1" s="1">
+      <x:c r="A4" s="23" t="inlineStr">
+        <x:is>
+          <x:t>unlock_stage</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B4" s="23" t="inlineStr">
+        <x:is>
+          <x:t>int</x:t>
+        </x:is>
       </x:c>
       <x:c r="C4" s="24" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D4" s="19" t="str">
-        <x:v>主线最高到达关</x:v>
-      </x:c>
-      <x:c r="E4" s="19" t="str">
-        <x:v>默认7。异空间开放门槛。调大更晚开放，调小更早开放；达到门槛仍需满足路线最低关卡和资源条件。正整数，不新增关卡内容。</x:v>
-      </x:c>
-      <x:c r="F4" s="19" t="str">
-        <x:v>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:v>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="inlineStr">
+        <x:is>
+          <x:t>主线最高到达关</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E4" s="23" t="inlineStr">
+        <x:is>
+          <x:t>默认7。异空间开放门槛。调大更晚开放，调小更早开放；达到门槛仍需满足路线最低关卡和资源条件。正整数，不新增关卡内容。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F4" s="23" t="inlineStr">
+        <x:is>
+          <x:t>正整数，有限且&lt;9e15；必须&gt;0；保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查</x:t>
+        </x:is>
       </x:c>
       <x:c r="G4" s="23" t="b">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
Refresh zero-ticket descriptions and remove redundant checks
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/hyperspace_config.xlsx
+++ b/space-battleship/config_excel/hyperspace_config.xlsx
@@ -691,7 +691,7 @@
       </c>
       <c r="E6" s="23" t="inlineStr">
         <is>
-          <t>默认10。在线异空间充能基础速度。调大更快攒票，调小更慢；受挂设及60关后补给倍率共同作用。随游戏时间推进，离线不补充。</t>
+          <t>默认10。在线异空间充能基础速度；当前手动与自动挑战票耗均为0，本值不影响入场成本。随游戏时间推进，离线不补充。</t>
         </is>
       </c>
       <c r="F6" s="23" t="inlineStr">
@@ -757,12 +757,12 @@
       </c>
       <c r="E8" s="23" t="inlineStr">
         <is>
-          <t>默认108000。手动票耗及自动票耗基数。调大每次消耗更多，调小更便宜；自动再乘B/(B+船员等级)，失败仅退实际已付票。例如B=20、等级20，自动票耗为此值的一半。</t>
+          <t>当前值为0；手动挑战和自动挑战均不消耗票。此字段保留为票耗配置入口，当前不按旧票耗基数或船员折扣收费。</t>
         </is>
       </c>
       <c r="F8" s="23" t="inlineStr">
         <is>
-          <t>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；&gt;0</t>
+          <t>保留当前JSON类型；数值有限；运行时C.number边界abs(value)&lt;9e15；相关跨字段约束必须导入和启动均检查；&gt;=0</t>
         </is>
       </c>
       <c r="G8" s="23" t="b">

</xml_diff>